<commit_message>
ordered max96717 v2, csi adpt for imx307, and bcm ecu reva
</commit_message>
<xml_diff>
--- a/1_BCM_ECU/3_BCM_ECU_revA/Project Outputs for BCM_ECU/BCM_ECU.xlsx
+++ b/1_BCM_ECU/3_BCM_ECU_revA/Project Outputs for BCM_ECU/BCM_ECU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\se097192\Documents\0_BRZ\BRZ_HARDWARE\1_BCM_ECU\3_BCM_ECU_revA\Project Outputs for BCM_ECU\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\se097192\Documents\0_BRZ\BRZ_HARDWARE_V2\1_BCM_ECU\3_BCM_ECU_revA\Project Outputs for BCM_ECU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0F156C5-F747-45B5-8488-35D3BFBA101F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E487588E-4C70-400D-947A-03994CCBB460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" xr2:uid="{D9E6F516-F670-479D-878A-2EBB97CA7047}"/>
+    <workbookView xWindow="-38520" yWindow="-3765" windowWidth="38640" windowHeight="21120" xr2:uid="{7CE6E4B5-DEBC-4686-9A7D-D0AA47A550C3}"/>
   </bookViews>
   <sheets>
     <sheet name="BCM_ECU" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="319">
   <si>
     <t>Line #</t>
   </si>
@@ -212,24 +212,24 @@
     <t>CMP-08246-004290-1</t>
   </si>
   <si>
+    <t>810-C5750X7R2A335K</t>
+  </si>
+  <si>
+    <t>CKG57NX5R1H226M500JH</t>
+  </si>
+  <si>
+    <t>CAP CER 22UF 50V X5R SMD</t>
+  </si>
+  <si>
+    <t>C64, C65, C110, C111</t>
+  </si>
+  <si>
+    <t>CMP-08246-005087-1</t>
+  </si>
+  <si>
     <t>Digikey</t>
   </si>
   <si>
-    <t>445-4524-1-ND</t>
-  </si>
-  <si>
-    <t>CKG57NX5R1H226M500JH</t>
-  </si>
-  <si>
-    <t>CAP CER 22UF 50V X5R SMD</t>
-  </si>
-  <si>
-    <t>C64, C65, C110, C111</t>
-  </si>
-  <si>
-    <t>CMP-08246-005087-1</t>
-  </si>
-  <si>
     <t>445-1655-1-ND</t>
   </si>
   <si>
@@ -245,369 +245,354 @@
     <t>CMP-14477-002774-2</t>
   </si>
   <si>
+    <t>963-HMK325B7105KN-T</t>
+  </si>
+  <si>
+    <t>C0805C103K2RACTU</t>
+  </si>
+  <si>
+    <t>CAP CER 10000PF 200V X7R 0805</t>
+  </si>
+  <si>
+    <t>C78, C86</t>
+  </si>
+  <si>
+    <t>CMP-2007-00259-2</t>
+  </si>
+  <si>
+    <t>KEMET</t>
+  </si>
+  <si>
+    <t>MAL215099913E3</t>
+  </si>
+  <si>
+    <t>Aluminum Electrolytic Capacitor, Polarized, Aluminum (wet), 100V, 20% +Tol, 20% -Tol, 470uF, Surface Mount, 7171</t>
+  </si>
+  <si>
+    <t>C88, C92</t>
+  </si>
+  <si>
+    <t>CMP-001-00064-1</t>
+  </si>
+  <si>
+    <t>Vishay BCcomponents</t>
+  </si>
+  <si>
+    <t>C3829592</t>
+  </si>
+  <si>
+    <t>12103D106KAT2A</t>
+  </si>
+  <si>
+    <t>General Purpose Ceramic Capacitor, 1210, 10uF, 10%, X5R, 15%, 25V</t>
+  </si>
+  <si>
+    <t>C96, C118</t>
+  </si>
+  <si>
+    <t>CMP-2000-05477-2</t>
+  </si>
+  <si>
+    <t>C1210C105J5RACTU</t>
+  </si>
+  <si>
+    <t>399-C1210C105J5RACTUCT-ND</t>
+  </si>
+  <si>
+    <t>MMSZ5242BT1G</t>
+  </si>
+  <si>
+    <t>Zener Voltage Regulator, 500 mW, 2-Pin SOD-123, Pb-Free, Tape and Reel</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>CMP-1060-00565-1</t>
+  </si>
+  <si>
+    <t>onsemi</t>
+  </si>
+  <si>
+    <t>58M9232</t>
+  </si>
+  <si>
+    <t>1N4148W-TP</t>
+  </si>
+  <si>
+    <t>DIODE GEN PURP 100V 150MA SOD123</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>CMP-2000-04993-2</t>
+  </si>
+  <si>
+    <t>MCC</t>
+  </si>
+  <si>
+    <t>51AH9840</t>
+  </si>
+  <si>
+    <t>ESDCAN02-2BWY</t>
+  </si>
+  <si>
+    <t>TVS DIODE 26.5V 44V SOT323-3</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>CMP-12225-000055-1</t>
+  </si>
+  <si>
+    <t>STMicroelectronics</t>
+  </si>
+  <si>
+    <t>03AJ0573</t>
+  </si>
+  <si>
+    <t>150066RG54050</t>
+  </si>
+  <si>
+    <t>Led, Red/Grn, 180Mcd/230Mcd, 624Nm/525Nm Rohs Compliant: Yes</t>
+  </si>
+  <si>
+    <t>D4, D5</t>
+  </si>
+  <si>
+    <t>CMP-004-00040-2</t>
+  </si>
+  <si>
+    <t>MM5Z3V3T1G</t>
+  </si>
+  <si>
+    <t>Zener Voltage Regulator, 500 mW, 2-Pin SOD-523, Pb-Free, Tape and Reel</t>
+  </si>
+  <si>
+    <t>D6_PWR_PROT_1, D6_PWR_PROT_2, D6_PWR_PROT_3, D6_PWR_PROT_4, D6_PWR_PROT_5, D8, D9_IO_CHECKER_0, D9_IO_CHECKER_1, D10_IO_CHECKER_0, D10_IO_CHECKER_1, D11_IO_CHECKER_0, D11_IO_CHECKER_1, D12_IO_CHECKER_0, D12_IO_CHECKER_1, D13_IO_CHECKER_0, D13_IO_CHECKER_1, D14_IO_CHECKER_0, D14_IO_CHECKER_1, D15_IO_CHECKER_0, D15_IO_CHECKER_1, D16_IO_CHECKER_0, D16_IO_CHECKER_1, D17_IO_CHECKER_0, D17_IO_CHECKER_1, D18_IO_CHECKER_0, D18_IO_CHECKER_1, D19_IO_CHECKER_0, D19_IO_CHECKER_1, D20_IO_CHECKER_0, D20_IO_CHECKER_1, D21_IO_CHECKER_0, D21_IO_CHECKER_1, D22_IO_CHECKER_0, D22_IO_CHECKER_1, D23, D26_ADC_0, D26_ADC_1, D27_ADC_0, D27_ADC_1, D28_ADC_0, D28_ADC_1, D29_ADC_0, D29_ADC_1, D30_ADC_0, D30_ADC_1, D31_ADC_0, D31_ADC_1, D32_ADC_0, D32_ADC_1, D33_ADC_0, D33_ADC_1, D34, D35, D36, D37, D38, D39, D40, D41_MOSFET_BANK_0, D41_MOSFET_BANK_1, D41_MOSFET_BANK_2, D41_MOSFET_BANK_3, D42_MOSFET_BANK_0, D42_MOSFET_BANK_1, D42_MOSFET_BANK_2, D42_MOSFET_BANK_3, D43_MOSFET_BANK_0, D43_MOSFET_BANK_1, D43_MOSFET_BANK_2, D43_MOSFET_BANK_3, D44_MOSFET_BANK_0, D44_MOSFET_BANK_1, D44_MOSFET_BANK_2, D44_MOSFET_BANK_3, D45, D46, D47</t>
+  </si>
+  <si>
+    <t>CMP-1060-00750-1</t>
+  </si>
+  <si>
+    <t>09R9519</t>
+  </si>
+  <si>
+    <t>SK34A-LTP</t>
+  </si>
+  <si>
+    <t>Rectifier Diode, Schottky, 1 Phase, 1 Element, 3A, 40V V(RRM), Silicon, DO-214AC</t>
+  </si>
+  <si>
+    <t>D7_BYPASS_0, D7_BYPASS_1, D7_BYPASS_2, D7_BYPASS_3</t>
+  </si>
+  <si>
+    <t>CMP-004-00058-2</t>
+  </si>
+  <si>
+    <t>SK34A-LTPMSDKR-ND</t>
+  </si>
+  <si>
+    <t>TVU1240R1ADG</t>
+  </si>
+  <si>
+    <t>D24, D25</t>
+  </si>
+  <si>
+    <t>CMP-004-00060-2</t>
+  </si>
+  <si>
+    <t>INPAQ TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>3526-TVU1240R1ADGCT-ND</t>
+  </si>
+  <si>
+    <t>0ZCH0075AF2E</t>
+  </si>
+  <si>
+    <t>PTC Thermistor</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>CMP-005-00028-2</t>
+  </si>
+  <si>
+    <t>Bel</t>
+  </si>
+  <si>
+    <t>530-0ZCH0075AF2E</t>
+  </si>
+  <si>
+    <t>0466003.NR</t>
+  </si>
+  <si>
+    <t>FUSE BOARD MNT 3A 32VAC/VDC 1206</t>
+  </si>
+  <si>
+    <t>F2_MOSFET_BANK_0, F2_MOSFET_BANK_1, F2_MOSFET_BANK_2, F2_MOSFET_BANK_3, F3_MOSFET_BANK_0, F3_MOSFET_BANK_1, F3_MOSFET_BANK_2, F3_MOSFET_BANK_3, F4_MOSFET_BANK_0, F4_MOSFET_BANK_1, F4_MOSFET_BANK_2, F4_MOSFET_BANK_3, F5_MOSFET_BANK_0, F5_MOSFET_BANK_1, F5_MOSFET_BANK_2, F5_MOSFET_BANK_3, F6_BYPASS_0, F6_BYPASS_1, F6_BYPASS_2, F6_BYPASS_3</t>
+  </si>
+  <si>
+    <t>CMP-08605-000054-1</t>
+  </si>
+  <si>
+    <t>Littelfuse</t>
+  </si>
+  <si>
+    <t>Arrow Electronics</t>
+  </si>
+  <si>
+    <t>MF-PSMF020X-2</t>
+  </si>
+  <si>
+    <t>PTC RESET FUSE 9V 200MA 0805</t>
+  </si>
+  <si>
+    <t>F7, F8, F9, F11, F13</t>
+  </si>
+  <si>
+    <t>CMP-07400-000005-1</t>
+  </si>
+  <si>
+    <t>Bourns</t>
+  </si>
+  <si>
+    <t>MF-PSMF020X-2CT-ND</t>
+  </si>
+  <si>
+    <t>BLM15PX601SN1D</t>
+  </si>
+  <si>
+    <t>Chip Ferrite Bead, 0402, 600Ω @ 100MHz, 0.23Ω, 25%, 900mA</t>
+  </si>
+  <si>
+    <t>FB1</t>
+  </si>
+  <si>
+    <t>CMP-0686-00252-4</t>
+  </si>
+  <si>
+    <t>490-9657-6-ND</t>
+  </si>
+  <si>
+    <t>776163-1</t>
+  </si>
+  <si>
+    <t>CONN HEADER R/A 35POS 4MM</t>
+  </si>
+  <si>
+    <t>J1, J2</t>
+  </si>
+  <si>
+    <t>CMP-03369-000154-1</t>
+  </si>
+  <si>
+    <t>TE Connectivity</t>
+  </si>
+  <si>
+    <t>3220-10-0300-00</t>
+  </si>
+  <si>
+    <t>CONN HEADER SMD 10POS 1.27MM</t>
+  </si>
+  <si>
+    <t>J4</t>
+  </si>
+  <si>
+    <t>CMP-001-0013-3</t>
+  </si>
+  <si>
+    <t>CNC Tech</t>
+  </si>
+  <si>
+    <t>1175-1629-ND</t>
+  </si>
+  <si>
+    <t>SRF4532-510Y</t>
+  </si>
+  <si>
+    <t>CMC 51UH 200MA 2LN 2KOHM SMD</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>CMP-07251-000006-1</t>
+  </si>
+  <si>
+    <t>63W2964</t>
+  </si>
+  <si>
+    <t>74435561100</t>
+  </si>
+  <si>
+    <t>L2, L4</t>
+  </si>
+  <si>
+    <t>CMP-0226-00001-2</t>
+  </si>
+  <si>
+    <t>Wurth Electronics</t>
+  </si>
+  <si>
+    <t>732-2167-6-ND</t>
+  </si>
+  <si>
+    <t>PM5433.302NLT</t>
+  </si>
+  <si>
+    <t>High Current Composite Inductor - PA5433.XXXNLT and PM5433.XXXNLT</t>
+  </si>
+  <si>
+    <t>L3</t>
+  </si>
+  <si>
+    <t>CMP-006-00032-1</t>
+  </si>
+  <si>
+    <t>Pulse</t>
+  </si>
+  <si>
+    <t>553-PM5433.302NLTCT-ND</t>
+  </si>
+  <si>
+    <t>SISH615ADN-T1-GE3</t>
+  </si>
+  <si>
+    <t>Trans MOSFET P-CH 20V 22.1A 8-Pin PowerPAK 1212 EP T/R</t>
+  </si>
+  <si>
+    <t>Q1, Q2, Q3, Q4, Q7_BYPASS_0, Q7_BYPASS_1, Q7_BYPASS_2, Q7_BYPASS_3</t>
+  </si>
+  <si>
+    <t>CMP-013-00018-2</t>
+  </si>
+  <si>
+    <t>BSS138W-7-F</t>
+  </si>
+  <si>
+    <t>N-Channel Enhancement Mode Mosfet, 50 V, 200 mA, -55 to 150 degC, 6-Pin SOT-323, RoHS, Tape and Reel</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>CMP-2000-05968-1</t>
+  </si>
+  <si>
+    <t>Diodes</t>
+  </si>
+  <si>
     <t>Future Electronics</t>
   </si>
   <si>
-    <t>2118828</t>
-  </si>
-  <si>
-    <t>C0805C103K2RACTU</t>
-  </si>
-  <si>
-    <t>CAP CER 10000PF 200V X7R 0805</t>
-  </si>
-  <si>
-    <t>C78, C86</t>
-  </si>
-  <si>
-    <t>CMP-2007-00259-2</t>
-  </si>
-  <si>
-    <t>KEMET</t>
-  </si>
-  <si>
-    <t>MAL215099913E3</t>
-  </si>
-  <si>
-    <t>Aluminum Electrolytic Capacitor, Polarized, Aluminum (wet), 100V, 20% +Tol, 20% -Tol, 470uF, Surface Mount, 7171</t>
-  </si>
-  <si>
-    <t>C88, C92</t>
-  </si>
-  <si>
-    <t>CMP-001-00064-1</t>
-  </si>
-  <si>
-    <t>Vishay BCcomponents</t>
-  </si>
-  <si>
-    <t>C3829592</t>
-  </si>
-  <si>
-    <t>12103D106KAT2A</t>
-  </si>
-  <si>
-    <t>General Purpose Ceramic Capacitor, 1210, 10uF, 10%, X5R, 15%, 25V</t>
-  </si>
-  <si>
-    <t>C96, C118</t>
-  </si>
-  <si>
-    <t>CMP-2000-05477-2</t>
-  </si>
-  <si>
-    <t>C1210C105J5RACTU</t>
-  </si>
-  <si>
-    <t>399-C1210C105J5RACTUCT-ND</t>
-  </si>
-  <si>
-    <t>MMSZ5242BT1G</t>
-  </si>
-  <si>
-    <t>Zener Voltage Regulator, 500 mW, 2-Pin SOD-123, Pb-Free, Tape and Reel</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>CMP-1060-00565-1</t>
-  </si>
-  <si>
-    <t>onsemi</t>
-  </si>
-  <si>
-    <t>58M9232</t>
-  </si>
-  <si>
-    <t>1N4148W-TP</t>
-  </si>
-  <si>
-    <t>DIODE GEN PURP 100V 150MA SOD123</t>
-  </si>
-  <si>
-    <t>D2</t>
-  </si>
-  <si>
-    <t>CMP-2000-04993-2</t>
-  </si>
-  <si>
-    <t>MCC</t>
-  </si>
-  <si>
-    <t>51AH9840</t>
-  </si>
-  <si>
-    <t>ESDCAN02-2BWY</t>
-  </si>
-  <si>
-    <t>TVS DIODE 26.5V 44V SOT323-3</t>
-  </si>
-  <si>
-    <t>D3</t>
-  </si>
-  <si>
-    <t>CMP-12225-000055-1</t>
-  </si>
-  <si>
-    <t>STMicroelectronics</t>
-  </si>
-  <si>
-    <t>03AJ0573</t>
-  </si>
-  <si>
-    <t>150066RG54050</t>
-  </si>
-  <si>
-    <t>Led, Red/Grn, 180Mcd/230Mcd, 624Nm/525Nm Rohs Compliant: Yes</t>
-  </si>
-  <si>
-    <t>D4, D5</t>
-  </si>
-  <si>
-    <t>CMP-004-00040-2</t>
-  </si>
-  <si>
-    <t>MM5Z3V3T1G</t>
-  </si>
-  <si>
-    <t>Zener Voltage Regulator, 500 mW, 2-Pin SOD-523, Pb-Free, Tape and Reel</t>
-  </si>
-  <si>
-    <t>D6_PWR_PROT_1, D6_PWR_PROT_2, D6_PWR_PROT_3, D6_PWR_PROT_4, D6_PWR_PROT_5, D8, D9_IO_CHECKER_0, D9_IO_CHECKER_1, D10_IO_CHECKER_0, D10_IO_CHECKER_1, D11_IO_CHECKER_0, D11_IO_CHECKER_1, D12_IO_CHECKER_0, D12_IO_CHECKER_1, D13_IO_CHECKER_0, D13_IO_CHECKER_1, D14_IO_CHECKER_0, D14_IO_CHECKER_1, D15_IO_CHECKER_0, D15_IO_CHECKER_1, D16_IO_CHECKER_0, D16_IO_CHECKER_1, D17_IO_CHECKER_0, D17_IO_CHECKER_1, D18_IO_CHECKER_0, D18_IO_CHECKER_1, D19_IO_CHECKER_0, D19_IO_CHECKER_1, D20_IO_CHECKER_0, D20_IO_CHECKER_1, D21_IO_CHECKER_0, D21_IO_CHECKER_1, D22_IO_CHECKER_0, D22_IO_CHECKER_1, D23, D26_ADC_0, D26_ADC_1, D27_ADC_0, D27_ADC_1, D28_ADC_0, D28_ADC_1, D29_ADC_0, D29_ADC_1, D30_ADC_0, D30_ADC_1, D31_ADC_0, D31_ADC_1, D32_ADC_0, D32_ADC_1, D33_ADC_0, D33_ADC_1, D34, D35, D36, D37, D38, D39, D40, D41_MOSFET_BANK_0, D41_MOSFET_BANK_1, D41_MOSFET_BANK_2, D41_MOSFET_BANK_3, D42_MOSFET_BANK_0, D42_MOSFET_BANK_1, D42_MOSFET_BANK_2, D42_MOSFET_BANK_3, D43_MOSFET_BANK_0, D43_MOSFET_BANK_1, D43_MOSFET_BANK_2, D43_MOSFET_BANK_3, D44_MOSFET_BANK_0, D44_MOSFET_BANK_1, D44_MOSFET_BANK_2, D44_MOSFET_BANK_3, D45, D46, D47</t>
-  </si>
-  <si>
-    <t>CMP-1060-00750-1</t>
-  </si>
-  <si>
-    <t>09R9519</t>
-  </si>
-  <si>
-    <t>SK34A-LTP</t>
-  </si>
-  <si>
-    <t>Rectifier Diode, Schottky, 1 Phase, 1 Element, 3A, 40V V(RRM), Silicon, DO-214AC</t>
-  </si>
-  <si>
-    <t>D7_BYPASS_0, D7_BYPASS_1, D7_BYPASS_2, D7_BYPASS_3</t>
-  </si>
-  <si>
-    <t>CMP-004-00058-2</t>
-  </si>
-  <si>
-    <t>C85269</t>
-  </si>
-  <si>
-    <t>TVU1240R1ADG</t>
-  </si>
-  <si>
-    <t>D24, D25</t>
-  </si>
-  <si>
-    <t>CMP-004-00060-2</t>
-  </si>
-  <si>
-    <t>INPAQ TECHNOLOGY</t>
-  </si>
-  <si>
-    <t>Unknown</t>
-  </si>
-  <si>
-    <t>3526-TVU1240R1ADGCT-ND</t>
-  </si>
-  <si>
-    <t>0ZCH0075AF2E</t>
-  </si>
-  <si>
-    <t>PTC Thermistor</t>
-  </si>
-  <si>
-    <t>F1</t>
-  </si>
-  <si>
-    <t>CMP-005-00028-2</t>
-  </si>
-  <si>
-    <t>Bel</t>
-  </si>
-  <si>
-    <t>530-0ZCH0075AF2E</t>
-  </si>
-  <si>
-    <t>0466003.NR</t>
-  </si>
-  <si>
-    <t>FUSE BOARD MNT 3A 32VAC/VDC 1206</t>
-  </si>
-  <si>
-    <t>F2_MOSFET_BANK_0, F2_MOSFET_BANK_1, F2_MOSFET_BANK_2, F2_MOSFET_BANK_3, F3_MOSFET_BANK_0, F3_MOSFET_BANK_1, F3_MOSFET_BANK_2, F3_MOSFET_BANK_3, F4_MOSFET_BANK_0, F4_MOSFET_BANK_1, F4_MOSFET_BANK_2, F4_MOSFET_BANK_3, F5_MOSFET_BANK_0, F5_MOSFET_BANK_1, F5_MOSFET_BANK_2, F5_MOSFET_BANK_3, F6_BYPASS_0, F6_BYPASS_1, F6_BYPASS_2, F6_BYPASS_3</t>
-  </si>
-  <si>
-    <t>CMP-08605-000054-1</t>
-  </si>
-  <si>
-    <t>Littelfuse</t>
-  </si>
-  <si>
-    <t>Arrow Electronics</t>
-  </si>
-  <si>
-    <t>MF-PSMF020X-2</t>
-  </si>
-  <si>
-    <t>PTC RESET FUSE 9V 200MA 0805</t>
-  </si>
-  <si>
-    <t>F7, F8</t>
-  </si>
-  <si>
-    <t>CMP-07400-000005-1</t>
-  </si>
-  <si>
-    <t>Bourns</t>
-  </si>
-  <si>
-    <t>652-MF-PSMF020X-2</t>
-  </si>
-  <si>
-    <t>MF-PSMF010X-2</t>
-  </si>
-  <si>
-    <t>PTC RESET FUSE 15V 100MA 0805</t>
-  </si>
-  <si>
-    <t>F9_MOSFET_BANK_0, F9_MOSFET_BANK_1, F9_MOSFET_BANK_2, F9_MOSFET_BANK_3, F10_ADC_0, F10_ADC_1, F11, F12_IO_CHECKER_0, F12_IO_CHECKER_1</t>
-  </si>
-  <si>
-    <t>CMP-07400-000017-1</t>
-  </si>
-  <si>
-    <t>87W5967</t>
-  </si>
-  <si>
-    <t>BLM15PX601SN1D</t>
-  </si>
-  <si>
-    <t>Chip Ferrite Bead, 0402, 600Ω @ 100MHz, 0.23Ω, 25%, 900mA</t>
-  </si>
-  <si>
-    <t>FB1</t>
-  </si>
-  <si>
-    <t>CMP-0686-00252-4</t>
-  </si>
-  <si>
-    <t>490-9657-1-ND</t>
-  </si>
-  <si>
-    <t>776163-1</t>
-  </si>
-  <si>
-    <t>CONN HEADER R/A 35POS 4MM</t>
-  </si>
-  <si>
-    <t>J1, J2</t>
-  </si>
-  <si>
-    <t>CMP-03369-000154-1</t>
-  </si>
-  <si>
-    <t>TE Connectivity</t>
-  </si>
-  <si>
-    <t>3220-10-0300-00</t>
-  </si>
-  <si>
-    <t>CONN HEADER SMD 10POS 1.27MM</t>
-  </si>
-  <si>
-    <t>J4</t>
-  </si>
-  <si>
-    <t>CMP-001-0013-3</t>
-  </si>
-  <si>
-    <t>CNC Tech</t>
-  </si>
-  <si>
-    <t>1175-1629-ND</t>
-  </si>
-  <si>
-    <t>SRF4532-510Y</t>
-  </si>
-  <si>
-    <t>CMC 51UH 200MA 2LN 2KOHM SMD</t>
-  </si>
-  <si>
-    <t>L1</t>
-  </si>
-  <si>
-    <t>CMP-07251-000006-1</t>
-  </si>
-  <si>
-    <t>63W2964</t>
-  </si>
-  <si>
-    <t>74435561100</t>
-  </si>
-  <si>
-    <t>L2, L4</t>
-  </si>
-  <si>
-    <t>CMP-0226-00001-2</t>
-  </si>
-  <si>
-    <t>Wurth Electronics</t>
-  </si>
-  <si>
-    <t>732-2167-1-ND</t>
-  </si>
-  <si>
-    <t>PM5433.302NLT</t>
-  </si>
-  <si>
-    <t>High Current Composite Inductor - PA5433.XXXNLT and PM5433.XXXNLT</t>
-  </si>
-  <si>
-    <t>L3</t>
-  </si>
-  <si>
-    <t>CMP-006-00032-1</t>
-  </si>
-  <si>
-    <t>Pulse</t>
-  </si>
-  <si>
-    <t>553-PM5433.302NLTCT-ND</t>
-  </si>
-  <si>
-    <t>SISH615ADN-T1-GE3</t>
-  </si>
-  <si>
-    <t>Trans MOSFET P-CH 20V 22.1A 8-Pin PowerPAK 1212 EP T/R</t>
-  </si>
-  <si>
-    <t>Q1, Q2, Q3, Q4, Q7_BYPASS_0, Q7_BYPASS_1, Q7_BYPASS_2, Q7_BYPASS_3</t>
-  </si>
-  <si>
-    <t>CMP-013-00018-2</t>
-  </si>
-  <si>
-    <t>BSS138W-7-F</t>
-  </si>
-  <si>
-    <t>N-Channel Enhancement Mode Mosfet, 50 V, 200 mA, -55 to 150 degC, 6-Pin SOT-323, RoHS, Tape and Reel</t>
-  </si>
-  <si>
-    <t>Q5</t>
-  </si>
-  <si>
-    <t>CMP-2000-05968-1</t>
-  </si>
-  <si>
-    <t>Diodes</t>
-  </si>
-  <si>
     <t>6104898</t>
   </si>
   <si>
@@ -626,7 +611,7 @@
     <t>Vishay</t>
   </si>
   <si>
-    <t>742-SUD80460E-GE3CT-ND</t>
+    <t>10AC9186</t>
   </si>
   <si>
     <t>SSM6L56FE,LM</t>
@@ -731,6 +716,9 @@
     <t>Molex</t>
   </si>
   <si>
+    <t>32T4523</t>
+  </si>
+  <si>
     <t>KXT331LHS</t>
   </si>
   <si>
@@ -902,6 +890,9 @@
     <t>CMP-07117-000003-1</t>
   </si>
   <si>
+    <t>698-CAT25256VI-GT3</t>
+  </si>
+  <si>
     <t>MCP23017-E/SS</t>
   </si>
   <si>
@@ -986,10 +977,7 @@
     <t>Abracon</t>
   </si>
   <si>
-    <t>Farnell</t>
-  </si>
-  <si>
-    <t>2101339</t>
+    <t>60R3974</t>
   </si>
   <si>
     <t>ECS-.327-12.5-1210-TR</t>
@@ -1007,7 +995,7 @@
     <t>ECS International</t>
   </si>
   <si>
-    <t>520-.327-12.5-1210T</t>
+    <t>XC2282CT-ND</t>
   </si>
 </sst>
 </file>
@@ -1403,8 +1391,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0976AADD-0684-41A3-8191-9D9A8BE8309C}">
-  <dimension ref="A1:O56"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7355EC9B-003C-4413-A470-4FD2177F1858}">
+  <dimension ref="A1:O55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="4" width="16" customWidth="1"/>
@@ -1509,10 +1497,10 @@
         <v>26</v>
       </c>
       <c r="N2" s="1">
-        <v>3.7000000000000002E-3</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="O2" s="1">
-        <v>0.38479999999999998</v>
+        <v>0.35360000000000003</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
@@ -1642,10 +1630,10 @@
         <v>45</v>
       </c>
       <c r="N5" s="1">
-        <v>0.23</v>
+        <v>0.16</v>
       </c>
       <c r="O5" s="1">
-        <v>0.46</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
@@ -1689,10 +1677,10 @@
         <v>52</v>
       </c>
       <c r="N6" s="1">
-        <v>1.62</v>
+        <v>1.69</v>
       </c>
       <c r="O6" s="1">
-        <v>19.440000000000001</v>
+        <v>20.28</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -1730,16 +1718,16 @@
         <v>24</v>
       </c>
       <c r="L7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M7" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M7" s="2" t="s">
-        <v>58</v>
-      </c>
       <c r="N7" s="1">
-        <v>1.47</v>
+        <v>1.2</v>
       </c>
       <c r="O7" s="1">
-        <v>14.72</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
@@ -1747,16 +1735,16 @@
         <v>15</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>31</v>
@@ -1771,13 +1759,13 @@
         <v>50</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>63</v>
@@ -1824,16 +1812,16 @@
         <v>24</v>
       </c>
       <c r="L9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="M9" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="N9" s="1">
-        <v>0.42</v>
+        <v>0.19400000000000001</v>
       </c>
       <c r="O9" s="1">
-        <v>2.1</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
@@ -1841,16 +1829,16 @@
         <v>15</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>31</v>
@@ -1862,10 +1850,10 @@
         <v>2</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>24</v>
@@ -1880,16 +1868,16 @@
         <v>15</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>20</v>
@@ -1901,10 +1889,10 @@
         <v>2</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>24</v>
@@ -1913,13 +1901,13 @@
         <v>25</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N11" s="1">
-        <v>5.36</v>
+        <v>5.17</v>
       </c>
       <c r="O11" s="1">
-        <v>10.72</v>
+        <v>10.34</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
@@ -1927,16 +1915,16 @@
         <v>15</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>84</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>44</v>
@@ -1948,19 +1936,19 @@
         <v>2</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J12" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M12" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="N12" s="1">
         <v>0.73</v>
@@ -1970,18 +1958,20 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B13" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>44</v>
@@ -1993,10 +1983,10 @@
         <v>1</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>24</v>
@@ -2005,7 +1995,7 @@
         <v>51</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N13" s="1">
         <v>2.1999999999999999E-2</v>
@@ -2015,18 +2005,20 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
+      <c r="A14" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B14" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>31</v>
@@ -2038,10 +2030,10 @@
         <v>1</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>24</v>
@@ -2050,7 +2042,7 @@
         <v>51</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N14" s="1">
         <v>2.1000000000000001E-2</v>
@@ -2060,18 +2052,20 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
+      <c r="A15" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B15" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>31</v>
@@ -2083,10 +2077,10 @@
         <v>1</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>24</v>
@@ -2095,13 +2089,13 @@
         <v>51</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="N15" s="1">
-        <v>8.5999999999999993E-2</v>
+        <v>0.06</v>
       </c>
       <c r="O15" s="1">
-        <v>8.5999999999999993E-2</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
@@ -2109,16 +2103,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>20</v>
@@ -2142,16 +2136,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>44</v>
@@ -2163,10 +2157,10 @@
         <v>77</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>24</v>
@@ -2175,7 +2169,7 @@
         <v>51</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="N17" s="1">
         <v>0.03</v>
@@ -2189,16 +2183,16 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>20</v>
@@ -2210,25 +2204,25 @@
         <v>4</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="N18" s="1">
-        <v>5.1999999999999998E-2</v>
+        <v>0.26</v>
       </c>
       <c r="O18" s="1">
-        <v>0.52</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
@@ -2236,16 +2230,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>20</v>
@@ -2257,19 +2251,19 @@
         <v>2</v>
       </c>
       <c r="I19" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="K19" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="J19" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="K19" s="2" t="s">
+      <c r="L19" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M19" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="N19" s="1">
         <v>0.25</v>
@@ -2279,18 +2273,20 @@
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
+      <c r="A20" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B20" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>128</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>20</v>
@@ -2302,10 +2298,10 @@
         <v>1</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>24</v>
@@ -2314,13 +2310,13 @@
         <v>33</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N20" s="1">
-        <v>0.24</v>
+        <v>0.21</v>
       </c>
       <c r="O20" s="1">
-        <v>0.24</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
@@ -2328,16 +2324,16 @@
         <v>15</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>134</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>31</v>
@@ -2349,25 +2345,25 @@
         <v>20</v>
       </c>
       <c r="I21" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="J21" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>136</v>
-      </c>
       <c r="M21" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N21" s="1">
-        <v>0.43070000000000003</v>
+        <v>0.40100000000000002</v>
       </c>
       <c r="O21" s="1">
-        <v>8.61</v>
+        <v>8.02</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
@@ -2375,16 +2371,16 @@
         <v>15</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>140</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>31</v>
@@ -2393,28 +2389,28 @@
         <v>21</v>
       </c>
       <c r="H22" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I22" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M22" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="J22" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L22" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>142</v>
-      </c>
       <c r="N22" s="1">
-        <v>0.3</v>
+        <v>0.29799999999999999</v>
       </c>
       <c r="O22" s="1">
-        <v>0.6</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
@@ -2422,16 +2418,16 @@
         <v>15</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>31</v>
@@ -2440,43 +2436,45 @@
         <v>21</v>
       </c>
       <c r="H23" s="1">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>141</v>
+        <v>32</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="M23" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="N23" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="O23" s="1">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="N23" s="1">
-        <v>0.22500000000000001</v>
-      </c>
-      <c r="O23" s="1">
-        <v>2.0299999999999998</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>151</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>31</v>
@@ -2485,28 +2483,28 @@
         <v>21</v>
       </c>
       <c r="H24" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>32</v>
+        <v>151</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>57</v>
+        <v>135</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="N24" s="1">
-        <v>0.1</v>
+        <v>10.63</v>
       </c>
       <c r="O24" s="1">
-        <v>0.1</v>
+        <v>21.27</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
@@ -2514,50 +2512,52 @@
         <v>15</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="D25" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="E25" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="F25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H25" s="1">
+        <v>1</v>
+      </c>
+      <c r="I25" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="F25" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H25" s="1">
-        <v>2</v>
-      </c>
-      <c r="I25" s="2" t="s">
+      <c r="J25" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M25" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="J25" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="M25" s="2" t="s">
-        <v>153</v>
-      </c>
       <c r="N25" s="1">
-        <v>11.68</v>
+        <v>0.81</v>
       </c>
       <c r="O25" s="1">
-        <v>23.36</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A26" s="1"/>
+      <c r="A26" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B26" s="2" t="s">
         <v>158</v>
       </c>
@@ -2571,7 +2571,7 @@
         <v>161</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>21</v>
@@ -2580,7 +2580,7 @@
         <v>1</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>162</v>
+        <v>140</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>158</v>
@@ -2589,61 +2589,63 @@
         <v>24</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="M26" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="N26" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="O26" s="1">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="N26" s="1">
-        <v>0.81</v>
-      </c>
-      <c r="O26" s="1">
-        <v>0.81</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A27" s="1"/>
-      <c r="B27" s="2" t="s">
+      <c r="C27" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="F27" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H27" s="1">
+        <v>2</v>
+      </c>
+      <c r="I27" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="J27" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M27" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="F27" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H27" s="1">
-        <v>1</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>168</v>
-      </c>
       <c r="N27" s="1">
-        <v>0.38</v>
+        <v>5.7</v>
       </c>
       <c r="O27" s="1">
-        <v>0.38</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
@@ -2651,10 +2653,10 @@
         <v>15</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>170</v>
@@ -2663,38 +2665,40 @@
         <v>171</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H28" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>172</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>24</v>
+        <v>122</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="M28" s="2" t="s">
         <v>173</v>
       </c>
       <c r="N28" s="1">
-        <v>5.7</v>
+        <v>3.85</v>
       </c>
       <c r="O28" s="1">
-        <v>11.4</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A29" s="1"/>
+      <c r="A29" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B29" s="2" t="s">
         <v>174</v>
       </c>
@@ -2714,106 +2718,108 @@
         <v>21</v>
       </c>
       <c r="H29" s="1">
-        <v>1</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="L29" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M29" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="N29" s="1">
-        <v>4.3899999999999997</v>
-      </c>
-      <c r="O29" s="1">
-        <v>4.3899999999999997</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="E30" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="F30" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H30" s="1">
+        <v>1</v>
+      </c>
+      <c r="I30" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="J30" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H30" s="1">
-        <v>8</v>
-      </c>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
+      <c r="M30" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="N30" s="1">
+        <v>0.158</v>
+      </c>
+      <c r="O30" s="1">
+        <v>0.158</v>
+      </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A31" s="1"/>
+      <c r="A31" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B31" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H31" s="1">
+        <v>2</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="J31" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H31" s="1">
-        <v>1</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>184</v>
-      </c>
       <c r="K31" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="N31" s="1">
-        <v>0.161</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="O31" s="1">
-        <v>0.161</v>
+        <v>2.2400000000000002</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
@@ -2821,16 +2827,16 @@
         <v>15</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>31</v>
@@ -2839,28 +2845,28 @@
         <v>21</v>
       </c>
       <c r="H32" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>24</v>
+        <v>122</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="N32" s="1">
-        <v>1.1200000000000001</v>
+        <v>0.32</v>
       </c>
       <c r="O32" s="1">
-        <v>2.2400000000000002</v>
+        <v>1.28</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
@@ -2868,7 +2874,7 @@
         <v>15</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>197</v>
@@ -2880,68 +2886,68 @@
         <v>199</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H33" s="1">
-        <v>4</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="L33" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="N33" s="1">
-        <v>0.32</v>
-      </c>
-      <c r="O33" s="1">
-        <v>1.28</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D34" s="2" t="s">
+      <c r="F34" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H34" s="1">
+        <v>4</v>
+      </c>
+      <c r="I34" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="J34" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M34" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H34" s="1">
-        <v>199</v>
-      </c>
-      <c r="I34" s="1"/>
-      <c r="J34" s="1"/>
-      <c r="K34" s="1"/>
-      <c r="L34" s="1"/>
-      <c r="M34" s="1"/>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
+      <c r="N34" s="1">
+        <v>0.11</v>
+      </c>
+      <c r="O34" s="1">
+        <v>0.44</v>
+      </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
@@ -2951,13 +2957,13 @@
         <v>205</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>15</v>
+        <v>206</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>44</v>
@@ -2966,10 +2972,10 @@
         <v>21</v>
       </c>
       <c r="H35" s="1">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>208</v>
+        <v>140</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>205</v>
@@ -2984,10 +2990,10 @@
         <v>209</v>
       </c>
       <c r="N35" s="1">
-        <v>0.13</v>
+        <v>3.5999999999999997E-2</v>
       </c>
       <c r="O35" s="1">
-        <v>0.52</v>
+        <v>0.504</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
@@ -3007,16 +3013,16 @@
         <v>213</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H36" s="1">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>141</v>
+        <v>214</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>210</v>
@@ -3025,139 +3031,143 @@
         <v>24</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N36" s="1">
-        <v>3.5999999999999997E-2</v>
+        <v>1.26</v>
       </c>
       <c r="O36" s="1">
-        <v>0.504</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A37" s="1"/>
+      <c r="A37" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B37" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H37" s="1">
-        <v>1</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="N37" s="1">
-        <v>1.26</v>
-      </c>
-      <c r="O37" s="1">
-        <v>1.26</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="I37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+      <c r="O37" s="1"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="F38" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H38" s="1">
+        <v>1</v>
+      </c>
+      <c r="I38" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="F38" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H38" s="1">
-        <v>13</v>
-      </c>
-      <c r="I38" s="1"/>
-      <c r="J38" s="1"/>
-      <c r="K38" s="1"/>
-      <c r="L38" s="1"/>
-      <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
-      <c r="O38" s="1"/>
+      <c r="J38" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="N38" s="1">
+        <v>1.18</v>
+      </c>
+      <c r="O38" s="1">
+        <v>1.18</v>
+      </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A39" s="1"/>
+      <c r="A39" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B39" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C39" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H39" s="1">
+        <v>3</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="J39" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H39" s="1">
-        <v>1</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="J39" s="2" t="s">
-        <v>225</v>
-      </c>
       <c r="K39" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>136</v>
+        <v>51</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="N39" s="1">
-        <v>0.90280000000000005</v>
+        <v>0.21299999999999999</v>
       </c>
       <c r="O39" s="1">
-        <v>0.90280000000000005</v>
+        <v>0.63900000000000001</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
@@ -3165,46 +3175,46 @@
         <v>15</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D40" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H40" s="1">
+        <v>23</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="J40" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="E40" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H40" s="1">
-        <v>3</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="K40" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="N40" s="1">
-        <v>0.21299999999999999</v>
+        <v>1.62</v>
       </c>
       <c r="O40" s="1">
-        <v>0.63900000000000001</v>
+        <v>37.26</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
@@ -3212,16 +3222,16 @@
         <v>15</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>44</v>
@@ -3230,45 +3240,37 @@
         <v>21</v>
       </c>
       <c r="H41" s="1">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="K41" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="L41" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="N41" s="1">
-        <v>1.62</v>
-      </c>
-      <c r="O41" s="1">
-        <v>37.26</v>
-      </c>
+      <c r="L41" s="1"/>
+      <c r="M41" s="1"/>
+      <c r="N41" s="1"/>
+      <c r="O41" s="1"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>44</v>
@@ -3277,37 +3279,45 @@
         <v>21</v>
       </c>
       <c r="H42" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L42" s="1"/>
-      <c r="M42" s="1"/>
-      <c r="N42" s="1"/>
-      <c r="O42" s="1"/>
+        <v>122</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="N42" s="1">
+        <v>3.79</v>
+      </c>
+      <c r="O42" s="1">
+        <v>26.53</v>
+      </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>44</v>
@@ -3316,46 +3326,48 @@
         <v>21</v>
       </c>
       <c r="H43" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>252</v>
+        <v>236</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>123</v>
+        <v>24</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="N43" s="1">
-        <v>3.22</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="O43" s="1">
-        <v>22.54</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
+      <c r="A44" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B44" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>21</v>
@@ -3363,30 +3375,18 @@
       <c r="H44" s="1">
         <v>1</v>
       </c>
-      <c r="I44" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="J44" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L44" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="M44" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="N44" s="1">
-        <v>1.19</v>
-      </c>
-      <c r="O44" s="1">
-        <v>1.19</v>
-      </c>
+      <c r="I44" s="1"/>
+      <c r="J44" s="1"/>
+      <c r="K44" s="1"/>
+      <c r="L44" s="1"/>
+      <c r="M44" s="1"/>
+      <c r="N44" s="1"/>
+      <c r="O44" s="1"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A45" s="1"/>
+      <c r="A45" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B45" s="2" t="s">
         <v>259</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>262</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>21</v>
@@ -3408,30 +3408,46 @@
       <c r="H45" s="1">
         <v>1</v>
       </c>
-      <c r="I45" s="1"/>
-      <c r="J45" s="1"/>
-      <c r="K45" s="1"/>
-      <c r="L45" s="1"/>
-      <c r="M45" s="1"/>
-      <c r="N45" s="1"/>
-      <c r="O45" s="1"/>
+      <c r="I45" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="N45" s="1">
+        <v>0.27800000000000002</v>
+      </c>
+      <c r="O45" s="1">
+        <v>0.27800000000000002</v>
+      </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A46" s="1"/>
+      <c r="A46" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B46" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>21</v>
@@ -3440,29 +3456,31 @@
         <v>1</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="K46" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>51</v>
+        <v>135</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="N46" s="1">
-        <v>0.28399999999999997</v>
+        <v>6.36</v>
       </c>
       <c r="O46" s="1">
-        <v>0.28399999999999997</v>
+        <v>6.36</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A47" s="1"/>
+      <c r="A47" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B47" s="2" t="s">
         <v>268</v>
       </c>
@@ -3485,7 +3503,7 @@
         <v>1</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J47" s="2" t="s">
         <v>268</v>
@@ -3494,34 +3512,36 @@
         <v>24</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>136</v>
+        <v>51</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="N47" s="1">
-        <v>6.86</v>
+        <v>0.27800000000000002</v>
       </c>
       <c r="O47" s="1">
-        <v>6.86</v>
+        <v>0.27800000000000002</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A48" s="1"/>
+      <c r="A48" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B48" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>21</v>
@@ -3530,43 +3550,45 @@
         <v>1</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>103</v>
+        <v>277</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>24</v>
+        <v>122</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="N48" s="1">
-        <v>0.28399999999999997</v>
+        <v>2.99</v>
       </c>
       <c r="O48" s="1">
-        <v>0.28399999999999997</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A49" s="1"/>
+      <c r="A49" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B49" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>21</v>
@@ -3575,70 +3597,72 @@
         <v>1</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>281</v>
+        <v>90</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>123</v>
+        <v>24</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="N49" s="1">
-        <v>2.89</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="O49" s="1">
-        <v>2.89</v>
+        <v>0.56999999999999995</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A50" s="1"/>
+      <c r="A50" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B50" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H50" s="1">
+        <v>2</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="J50" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H50" s="1">
-        <v>1</v>
-      </c>
-      <c r="I50" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="J50" s="2" t="s">
-        <v>283</v>
-      </c>
       <c r="K50" s="2" t="s">
         <v>24</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>136</v>
+        <v>289</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="N50" s="1">
-        <v>0.21840000000000001</v>
+        <v>1.33</v>
       </c>
       <c r="O50" s="1">
-        <v>0.21840000000000001</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
@@ -3646,64 +3670,66 @@
         <v>15</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="F51" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H51" s="1">
+        <v>1</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M51" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="N51" s="1">
+        <v>3.73</v>
+      </c>
+      <c r="O51" s="1">
+        <v>3.73</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H51" s="1">
-        <v>2</v>
-      </c>
-      <c r="I51" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="J51" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="K51" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L51" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="M51" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="N51" s="1">
-        <v>1.33</v>
-      </c>
-      <c r="O51" s="1">
-        <v>2.66</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A52" s="1"/>
-      <c r="B52" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>21</v>
@@ -3712,40 +3738,42 @@
         <v>1</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>24</v>
+        <v>122</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="N52" s="1">
-        <v>3.91</v>
+        <v>2.5299999999999998</v>
       </c>
       <c r="O52" s="1">
-        <v>3.91</v>
+        <v>2.5299999999999998</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A53" s="1"/>
+      <c r="A53" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B53" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>44</v>
@@ -3754,28 +3782,28 @@
         <v>21</v>
       </c>
       <c r="H53" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>281</v>
+        <v>305</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>123</v>
+        <v>24</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>57</v>
+        <v>183</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="N53" s="1">
-        <v>2.3199999999999998</v>
+        <v>0.67</v>
       </c>
       <c r="O53" s="1">
-        <v>2.3199999999999998</v>
+        <v>4.6900000000000004</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
@@ -3783,16 +3811,16 @@
         <v>15</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>44</v>
@@ -3801,46 +3829,48 @@
         <v>21</v>
       </c>
       <c r="H54" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>24</v>
+        <v>122</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="N54" s="1">
-        <v>0.67</v>
+        <v>0.434</v>
       </c>
       <c r="O54" s="1">
-        <v>4.6900000000000004</v>
+        <v>0.434</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A55" s="1"/>
+      <c r="A55" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="B55" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>21</v>
@@ -3849,69 +3879,24 @@
         <v>1</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>123</v>
+        <v>24</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>315</v>
+        <v>62</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="N55" s="1">
-        <v>0.38134000000000001</v>
+        <v>1.31</v>
       </c>
       <c r="O55" s="1">
-        <v>0.38134000000000001</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A56" s="1"/>
-      <c r="B56" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H56" s="1">
-        <v>1</v>
-      </c>
-      <c r="I56" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="J56" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="K56" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="M56" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="N56" s="1">
-        <v>1.31</v>
-      </c>
-      <c r="O56" s="1">
         <v>1.31</v>
       </c>
     </row>

</xml_diff>